<commit_message>
Record the picker click follow-up on Bugs row 282 and add its QA step
</commit_message>
<xml_diff>
--- a/docs/qa/QA_Bug_Fix_Testing.xlsx
+++ b/docs/qa/QA_Bug_Fix_Testing.xlsx
@@ -8896,7 +8896,10 @@
 5. Pick a long title, close the list, then hover the closed field.
 PASS: the full title shows steadily over the field.
 6. Open a run's history and repeat step 2 in both searchable filter pickers.
-PASS: same steady behaviour.</t>
+PASS: same steady behaviour.
+7. Pick a work item, then click anywhere on the field again (not only the arrow).
+PASS: the list opens straight away, so you can change to another work item.
+FAIL: nothing happens until you click somewhere else first or on the arrow.</t>
         </is>
       </c>
       <c r="I145" s="11" t="inlineStr">

</xml_diff>